<commit_message>
Component Placement Finalised, Starting Traces
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCBDEDD-5EC2-482B-B1C2-52D271805686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete Components" sheetId="1" r:id="rId1"/>
@@ -2447,6 +2447,59 @@
         <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF0563C1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2823,59 +2876,6 @@
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF0563C1"/>
-        <name val="Aptos Narrow"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2890,7 +2890,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K88" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K88" dataDxfId="16">
   <autoFilter ref="A1:K88" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="9">
       <filters>
@@ -2945,39 +2945,39 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Part Number" totalsRowLabel="3053 RD005" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Description" totalsRowLabel="20 AWG stranded red hook-up wire, 100 ft" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Manufacturer" totalsRowLabel="Alpha Wire" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Package" totalsRowLabel="N/A (bulk wire)" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Reference" totalsRowLabel="Fan and higher-current power wiring" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Qty" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Value" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{E789B1A8-406D-4F05-B177-7BF1F8F46C67}" name="Price(ZAR)" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Price Total" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Part Number" totalsRowLabel="3053 RD005" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Description" totalsRowLabel="20 AWG stranded red hook-up wire, 100 ft" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Manufacturer" totalsRowLabel="Alpha Wire" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Package" totalsRowLabel="N/A (bulk wire)" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Reference" totalsRowLabel="Fan and higher-current power wiring" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Qty" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Value" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{E789B1A8-406D-4F05-B177-7BF1F8F46C67}" name="Price(ZAR)" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Price Total" dataDxfId="7">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Qty]]*Table1[[#This Row],[Price(ZAR)]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="URL" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{59E2DE82-C8B4-4A42-87E4-805120F75DED}" name="KiCAD Assinged" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="URL" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{59E2DE82-C8B4-4A42-87E4-805120F75DED}" name="KiCAD Assinged" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7FDA6C1D-3E6A-45D5-B253-73D956697A60}" name="Table2" displayName="Table2" ref="A1:K51" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7FDA6C1D-3E6A-45D5-B253-73D956697A60}" name="Table2" displayName="Table2" ref="A1:K51" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29" totalsRowBorderDxfId="28">
   <autoFilter ref="A1:K51" xr:uid="{7FDA6C1D-3E6A-45D5-B253-73D956697A60}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0CA6AB1F-FAEE-4392-AA41-0547BB67F522}" name="Part Number" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{D1B2FCF2-7C8E-4E17-88C3-6184D268B2E6}" name="Description" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{6EDF6968-E12D-4739-A5C2-14BD1DDE85B1}" name="Manufacturer" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{91D4675B-E889-479C-BCA2-FCD90F4B4311}" name="Package" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{6306450D-9B29-4FAC-8DA3-7C18E1DB47F2}" name="Reference" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{5BC18179-D33D-4C57-8483-D34DFDC0DDEE}" name="Qty" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{C96A91E4-1884-430F-BAAA-56C1AF3B2686}" name="Value" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{B245D206-F331-43D5-B166-CB455F997AAE}" name="Price(ZAR)" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{9D5CA9D5-EE1B-41F5-992C-F9BF3DDC22A4}" name="Price Total" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{30D14786-057F-44B2-84ED-65CB7BB0C8A4}" name="URL" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{BE90A2EC-EC08-45A1-9554-65BAD2B399DB}" name="KiCAD Assinged" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{0CA6AB1F-FAEE-4392-AA41-0547BB67F522}" name="Part Number" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D1B2FCF2-7C8E-4E17-88C3-6184D268B2E6}" name="Description" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{6EDF6968-E12D-4739-A5C2-14BD1DDE85B1}" name="Manufacturer" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{91D4675B-E889-479C-BCA2-FCD90F4B4311}" name="Package" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{6306450D-9B29-4FAC-8DA3-7C18E1DB47F2}" name="Reference" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{5BC18179-D33D-4C57-8483-D34DFDC0DDEE}" name="Qty" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{C96A91E4-1884-430F-BAAA-56C1AF3B2686}" name="Value" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{B245D206-F331-43D5-B166-CB455F997AAE}" name="Price(ZAR)" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{9D5CA9D5-EE1B-41F5-992C-F9BF3DDC22A4}" name="Price Total" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{30D14786-057F-44B2-84ED-65CB7BB0C8A4}" name="URL" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{BE90A2EC-EC08-45A1-9554-65BAD2B399DB}" name="KiCAD Assinged" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Started equaliser PCB traces, need to check trace widths all round
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karlh\SkripsieProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCBDEDD-5EC2-482B-B1C2-52D271805686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A51ED8-ED27-40A7-98A3-FFB6C03B9B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7376,7 +7376,7 @@
       <c r="I36" s="24">
         <v>39.499900000000004</v>
       </c>
-      <c r="J36" s="30" t="s">
+      <c r="J36" s="25" t="s">
         <v>146</v>
       </c>
       <c r="K36" s="35"/>
@@ -7897,10 +7897,11 @@
     <hyperlink ref="J5" r:id="rId4" xr:uid="{773042D7-8C07-4F93-B732-FE2F9730B5C0}"/>
     <hyperlink ref="J23" r:id="rId5" xr:uid="{CD6EB69B-7D33-4CB3-B15C-F9C722EF19D2}"/>
     <hyperlink ref="J37" r:id="rId6" xr:uid="{4CFB475E-196C-4517-A456-D04BACC184B3}"/>
+    <hyperlink ref="J36" r:id="rId7" xr:uid="{0E20F516-3740-41B0-8214-9850C4D869D3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>